<commit_message>
Datos y alertas 2026-07-03
</commit_message>
<xml_diff>
--- a/alertas/alertas_2026-07-02.xlsx
+++ b/alertas/alertas_2026-07-02.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="38">
   <si>
     <t>Fecha</t>
   </si>
@@ -31,25 +31,49 @@
     <t>Unidad</t>
   </si>
   <si>
+    <t>02/07/2026 05:55</t>
+  </si>
+  <si>
+    <t>heladera BM reactivos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ambiente </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> °C</t>
+  </si>
+  <si>
+    <t>02/07/2026 05:46</t>
+  </si>
+  <si>
+    <t>heladera BM muestras</t>
+  </si>
+  <si>
+    <t>ambiente</t>
+  </si>
+  <si>
+    <t>02/07/2026 05:39</t>
+  </si>
+  <si>
+    <t>02/07/2026 05:31</t>
+  </si>
+  <si>
+    <t>02/07/2026 05:24</t>
+  </si>
+  <si>
+    <t>02/07/2026 05:16</t>
+  </si>
+  <si>
+    <t>02/07/2026 05:07</t>
+  </si>
+  <si>
+    <t>02/07/2026 05:00</t>
+  </si>
+  <si>
     <t>02/07/2026 04:52</t>
   </si>
   <si>
-    <t>heladera BM reactivos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ambiente </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> °C</t>
-  </si>
-  <si>
     <t>02/07/2026 04:45</t>
-  </si>
-  <si>
-    <t>heladera BM muestras</t>
-  </si>
-  <si>
-    <t>ambiente</t>
   </si>
   <si>
     <t>02/07/2026 04:36</t>
@@ -477,7 +501,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="4" width="20" customWidth="1"/>
@@ -680,10 +704,10 @@
         <v>21</v>
       </c>
       <c r="C12" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="D12" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E12">
         <v>26</v>
@@ -697,10 +721,10 @@
         <v>22</v>
       </c>
       <c r="C13" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D13" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E13">
         <v>26</v>
@@ -717,35 +741,35 @@
         <v>7</v>
       </c>
       <c r="D14" t="s">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="E14">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="F14" t="s">
-        <v>25</v>
+        <v>9</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C15" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D15" t="s">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="E15">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="F15" t="s">
-        <v>25</v>
+        <v>9</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C16" t="s">
         <v>7</v>
@@ -754,15 +778,15 @@
         <v>8</v>
       </c>
       <c r="E16">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="F16" t="s">
-        <v>25</v>
+        <v>9</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C17" t="s">
         <v>11</v>
@@ -779,16 +803,16 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C18" t="s">
         <v>7</v>
       </c>
       <c r="D18" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="E18">
-        <v>-15</v>
+        <v>26</v>
       </c>
       <c r="F18" t="s">
         <v>9</v>
@@ -796,18 +820,154 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>28</v>
+      </c>
+      <c r="C19" t="s">
+        <v>11</v>
+      </c>
+      <c r="D19" t="s">
+        <v>12</v>
+      </c>
+      <c r="E19">
+        <v>26</v>
+      </c>
+      <c r="F19" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
         <v>29</v>
       </c>
-      <c r="C19" t="s">
-        <v>7</v>
-      </c>
-      <c r="D19" t="s">
-        <v>26</v>
-      </c>
-      <c r="E19">
+      <c r="C20" t="s">
+        <v>11</v>
+      </c>
+      <c r="D20" t="s">
+        <v>12</v>
+      </c>
+      <c r="E20">
+        <v>26</v>
+      </c>
+      <c r="F20" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>30</v>
+      </c>
+      <c r="C21" t="s">
+        <v>7</v>
+      </c>
+      <c r="D21" t="s">
+        <v>8</v>
+      </c>
+      <c r="E21">
+        <v>26</v>
+      </c>
+      <c r="F21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>31</v>
+      </c>
+      <c r="C22" t="s">
+        <v>7</v>
+      </c>
+      <c r="D22" t="s">
+        <v>32</v>
+      </c>
+      <c r="E22">
+        <v>10</v>
+      </c>
+      <c r="F22" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>31</v>
+      </c>
+      <c r="C23" t="s">
+        <v>7</v>
+      </c>
+      <c r="D23" t="s">
+        <v>34</v>
+      </c>
+      <c r="E23">
+        <v>10</v>
+      </c>
+      <c r="F23" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>31</v>
+      </c>
+      <c r="C24" t="s">
+        <v>7</v>
+      </c>
+      <c r="D24" t="s">
+        <v>8</v>
+      </c>
+      <c r="E24">
+        <v>10</v>
+      </c>
+      <c r="F24" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>35</v>
+      </c>
+      <c r="C25" t="s">
+        <v>11</v>
+      </c>
+      <c r="D25" t="s">
+        <v>12</v>
+      </c>
+      <c r="E25">
+        <v>26</v>
+      </c>
+      <c r="F25" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>36</v>
+      </c>
+      <c r="C26" t="s">
+        <v>7</v>
+      </c>
+      <c r="D26" t="s">
+        <v>34</v>
+      </c>
+      <c r="E26">
         <v>-15</v>
       </c>
-      <c r="F19" t="s">
+      <c r="F26" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>37</v>
+      </c>
+      <c r="C27" t="s">
+        <v>7</v>
+      </c>
+      <c r="D27" t="s">
+        <v>34</v>
+      </c>
+      <c r="E27">
+        <v>-15</v>
+      </c>
+      <c r="F27" t="s">
         <v>9</v>
       </c>
     </row>

</xml_diff>